<commit_message>
Updated upload functions for reports
</commit_message>
<xml_diff>
--- a/data/uploads/ahd_screening.xlsx
+++ b/data/uploads/ahd_screening.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/innocentwowa/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/innocentwowa/Downloads/MaHIS dataset reports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6CB7607-101F-7E4A-990B-06185D533DEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F2CCC32-5783-C04F-AFD3-80F7ED3CE02B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="19880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1059" uniqueCount="734">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1203" uniqueCount="736">
   <si>
     <t>name</t>
   </si>
@@ -589,9 +589,6 @@
     <t>ahd_screening</t>
   </si>
   <si>
-    <t>ADVANCE HIV DISEASE QUARTERY REPORT</t>
-  </si>
-  <si>
     <t>period</t>
   </si>
   <si>
@@ -2243,17 +2240,33 @@
   </si>
   <si>
     <t>Zovirax</t>
+  </si>
+  <si>
+    <t>programs</t>
+  </si>
+  <si>
+    <t>Advanced HIV Disease Register – Facility Monthly Report</t>
+  </si>
+  <si>
+    <t>*AHD</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -2352,35 +2365,36 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -17120,7 +17134,9 @@
     <col min="1" max="1" width="31" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
     <col min="3" max="3" width="13.6640625" customWidth="1"/>
-    <col min="4" max="23" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.5" customWidth="1"/>
+    <col min="6" max="23" width="10.83203125" customWidth="1"/>
     <col min="24" max="26" width="10.5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -17205,8 +17221,12 @@
       <c r="C2" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
+      <c r="D2" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
@@ -17236,8 +17256,12 @@
       <c r="C3" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
+      <c r="D3" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
@@ -17267,8 +17291,12 @@
       <c r="C4" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
+      <c r="D4" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
@@ -17298,8 +17326,12 @@
       <c r="C5" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
+      <c r="D5" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
@@ -17329,8 +17361,12 @@
       <c r="C6" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
+      <c r="D6" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F6" s="1"/>
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
@@ -17360,8 +17396,12 @@
       <c r="C7" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
+      <c r="D7" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
@@ -17391,8 +17431,12 @@
       <c r="C8" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
+      <c r="D8" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
@@ -17422,8 +17466,12 @@
       <c r="C9" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D9" s="1"/>
-      <c r="E9" s="1"/>
+      <c r="D9" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
@@ -17453,8 +17501,12 @@
       <c r="C10" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
+      <c r="D10" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
@@ -17484,8 +17536,12 @@
       <c r="C11" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
+      <c r="D11" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
@@ -17515,8 +17571,12 @@
       <c r="C12" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
+      <c r="D12" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
@@ -17546,8 +17606,12 @@
       <c r="C13" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
+      <c r="D13" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
@@ -17577,8 +17641,12 @@
       <c r="C14" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
+      <c r="D14" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
@@ -17608,8 +17676,12 @@
       <c r="C15" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
+      <c r="D15" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
@@ -17639,8 +17711,12 @@
       <c r="C16" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
+      <c r="D16" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
@@ -17670,8 +17746,12 @@
       <c r="C17" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
+      <c r="D17" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
@@ -17701,8 +17781,12 @@
       <c r="C18" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
+      <c r="D18" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
@@ -17732,8 +17816,12 @@
       <c r="C19" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
+      <c r="D19" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
@@ -17763,8 +17851,12 @@
       <c r="C20" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
+      <c r="D20" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
@@ -17794,8 +17886,12 @@
       <c r="C21" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
+      <c r="D21" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
@@ -17825,8 +17921,12 @@
       <c r="C22" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
+      <c r="D22" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
@@ -17856,8 +17956,12 @@
       <c r="C23" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
+      <c r="D23" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
@@ -17887,8 +17991,12 @@
       <c r="C24" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
+      <c r="D24" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
@@ -17918,8 +18026,12 @@
       <c r="C25" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
+      <c r="D25" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
@@ -17949,8 +18061,12 @@
       <c r="C26" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D26" s="1"/>
-      <c r="E26" s="1"/>
+      <c r="D26" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
@@ -17980,8 +18096,12 @@
       <c r="C27" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D27" s="1"/>
-      <c r="E27" s="1"/>
+      <c r="D27" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
@@ -18011,8 +18131,12 @@
       <c r="C28" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D28" s="1"/>
-      <c r="E28" s="1"/>
+      <c r="D28" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
@@ -18042,8 +18166,12 @@
       <c r="C29" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D29" s="1"/>
-      <c r="E29" s="1"/>
+      <c r="D29" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
@@ -18073,8 +18201,12 @@
       <c r="C30" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D30" s="1"/>
-      <c r="E30" s="1"/>
+      <c r="D30" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
@@ -18104,8 +18236,12 @@
       <c r="C31" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D31" s="1"/>
-      <c r="E31" s="1"/>
+      <c r="D31" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F31" s="1"/>
       <c r="G31" s="1"/>
       <c r="H31" s="1"/>
@@ -18135,8 +18271,12 @@
       <c r="C32" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D32" s="1"/>
-      <c r="E32" s="1"/>
+      <c r="D32" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F32" s="1"/>
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
@@ -18166,8 +18306,12 @@
       <c r="C33" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D33" s="1"/>
-      <c r="E33" s="1"/>
+      <c r="D33" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
@@ -18197,8 +18341,12 @@
       <c r="C34" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D34" s="1"/>
-      <c r="E34" s="1"/>
+      <c r="D34" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F34" s="1"/>
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
@@ -18228,8 +18376,12 @@
       <c r="C35" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D35" s="1"/>
-      <c r="E35" s="1"/>
+      <c r="D35" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F35" s="1"/>
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
@@ -18259,8 +18411,12 @@
       <c r="C36" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D36" s="1"/>
-      <c r="E36" s="1"/>
+      <c r="D36" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F36" s="1"/>
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
@@ -18290,8 +18446,12 @@
       <c r="C37" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D37" s="1"/>
-      <c r="E37" s="1"/>
+      <c r="D37" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
@@ -18321,8 +18481,12 @@
       <c r="C38" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D38" s="1"/>
-      <c r="E38" s="1"/>
+      <c r="D38" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F38" s="1"/>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
@@ -18352,8 +18516,12 @@
       <c r="C39" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D39" s="1"/>
-      <c r="E39" s="1"/>
+      <c r="D39" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F39" s="1"/>
       <c r="G39" s="1"/>
       <c r="H39" s="1"/>
@@ -18383,8 +18551,12 @@
       <c r="C40" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D40" s="1"/>
-      <c r="E40" s="1"/>
+      <c r="D40" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F40" s="1"/>
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
@@ -18414,8 +18586,12 @@
       <c r="C41" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D41" s="1"/>
-      <c r="E41" s="1"/>
+      <c r="D41" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F41" s="1"/>
       <c r="G41" s="1"/>
       <c r="H41" s="1"/>
@@ -18445,8 +18621,12 @@
       <c r="C42" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D42" s="1"/>
-      <c r="E42" s="1"/>
+      <c r="D42" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F42" s="1"/>
       <c r="G42" s="1"/>
       <c r="H42" s="1"/>
@@ -18476,8 +18656,12 @@
       <c r="C43" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D43" s="1"/>
-      <c r="E43" s="1"/>
+      <c r="D43" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F43" s="1"/>
       <c r="G43" s="1"/>
       <c r="H43" s="1"/>
@@ -18507,8 +18691,12 @@
       <c r="C44" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D44" s="1"/>
-      <c r="E44" s="1"/>
+      <c r="D44" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F44" s="1"/>
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
@@ -18538,8 +18726,12 @@
       <c r="C45" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D45" s="1"/>
-      <c r="E45" s="1"/>
+      <c r="D45" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F45" s="1"/>
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
@@ -18569,8 +18761,12 @@
       <c r="C46" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D46" s="1"/>
-      <c r="E46" s="1"/>
+      <c r="D46" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F46" s="1"/>
       <c r="G46" s="1"/>
       <c r="H46" s="1"/>
@@ -18600,8 +18796,12 @@
       <c r="C47" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D47" s="1"/>
-      <c r="E47" s="1"/>
+      <c r="D47" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F47" s="1"/>
       <c r="G47" s="1"/>
       <c r="H47" s="1"/>
@@ -18631,8 +18831,12 @@
       <c r="C48" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D48" s="1"/>
-      <c r="E48" s="1"/>
+      <c r="D48" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F48" s="1"/>
       <c r="G48" s="1"/>
       <c r="H48" s="1"/>
@@ -18662,8 +18866,12 @@
       <c r="C49" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D49" s="1"/>
-      <c r="E49" s="1"/>
+      <c r="D49" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F49" s="1"/>
       <c r="G49" s="1"/>
       <c r="H49" s="1"/>
@@ -18693,8 +18901,12 @@
       <c r="C50" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D50" s="1"/>
-      <c r="E50" s="1"/>
+      <c r="D50" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F50" s="1"/>
       <c r="G50" s="1"/>
       <c r="H50" s="1"/>
@@ -18724,8 +18936,12 @@
       <c r="C51" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D51" s="1"/>
-      <c r="E51" s="1"/>
+      <c r="D51" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F51" s="1"/>
       <c r="G51" s="1"/>
       <c r="H51" s="1"/>
@@ -18755,8 +18971,12 @@
       <c r="C52" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D52" s="1"/>
-      <c r="E52" s="1"/>
+      <c r="D52" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F52" s="1"/>
       <c r="G52" s="1"/>
       <c r="H52" s="1"/>
@@ -18786,8 +19006,12 @@
       <c r="C53" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D53" s="1"/>
-      <c r="E53" s="1"/>
+      <c r="D53" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F53" s="1"/>
       <c r="G53" s="1"/>
       <c r="H53" s="1"/>
@@ -18817,8 +19041,12 @@
       <c r="C54" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D54" s="1"/>
-      <c r="E54" s="1"/>
+      <c r="D54" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F54" s="1"/>
       <c r="G54" s="1"/>
       <c r="H54" s="1"/>
@@ -18848,8 +19076,12 @@
       <c r="C55" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D55" s="1"/>
-      <c r="E55" s="1"/>
+      <c r="D55" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F55" s="1"/>
       <c r="G55" s="1"/>
       <c r="H55" s="1"/>
@@ -18879,8 +19111,12 @@
       <c r="C56" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D56" s="1"/>
-      <c r="E56" s="1"/>
+      <c r="D56" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F56" s="1"/>
       <c r="G56" s="1"/>
       <c r="H56" s="1"/>
@@ -18910,8 +19146,12 @@
       <c r="C57" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D57" s="1"/>
-      <c r="E57" s="1"/>
+      <c r="D57" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F57" s="1"/>
       <c r="G57" s="1"/>
       <c r="H57" s="1"/>
@@ -18941,8 +19181,12 @@
       <c r="C58" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D58" s="1"/>
-      <c r="E58" s="1"/>
+      <c r="D58" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F58" s="1"/>
       <c r="G58" s="1"/>
       <c r="H58" s="1"/>
@@ -18972,8 +19216,12 @@
       <c r="C59" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D59" s="1"/>
-      <c r="E59" s="1"/>
+      <c r="D59" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F59" s="1"/>
       <c r="G59" s="1"/>
       <c r="H59" s="1"/>
@@ -19003,8 +19251,12 @@
       <c r="C60" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D60" s="1"/>
-      <c r="E60" s="1"/>
+      <c r="D60" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F60" s="1"/>
       <c r="G60" s="1"/>
       <c r="H60" s="1"/>
@@ -19034,8 +19286,12 @@
       <c r="C61" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D61" s="1"/>
-      <c r="E61" s="1"/>
+      <c r="D61" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F61" s="1"/>
       <c r="G61" s="1"/>
       <c r="H61" s="1"/>
@@ -19065,8 +19321,12 @@
       <c r="C62" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D62" s="1"/>
-      <c r="E62" s="1"/>
+      <c r="D62" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F62" s="1"/>
       <c r="G62" s="1"/>
       <c r="H62" s="1"/>
@@ -19096,8 +19356,12 @@
       <c r="C63" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D63" s="1"/>
-      <c r="E63" s="1"/>
+      <c r="D63" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F63" s="1"/>
       <c r="G63" s="1"/>
       <c r="H63" s="1"/>
@@ -19127,8 +19391,12 @@
       <c r="C64" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D64" s="1"/>
-      <c r="E64" s="1"/>
+      <c r="D64" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E64" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F64" s="1"/>
       <c r="G64" s="1"/>
       <c r="H64" s="1"/>
@@ -19158,8 +19426,12 @@
       <c r="C65" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D65" s="1"/>
-      <c r="E65" s="1"/>
+      <c r="D65" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F65" s="1"/>
       <c r="G65" s="1"/>
       <c r="H65" s="1"/>
@@ -19189,8 +19461,12 @@
       <c r="C66" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D66" s="1"/>
-      <c r="E66" s="1"/>
+      <c r="D66" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E66" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F66" s="1"/>
       <c r="G66" s="1"/>
       <c r="H66" s="1"/>
@@ -19220,8 +19496,12 @@
       <c r="C67" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D67" s="1"/>
-      <c r="E67" s="1"/>
+      <c r="D67" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E67" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F67" s="1"/>
       <c r="G67" s="1"/>
       <c r="H67" s="1"/>
@@ -19251,8 +19531,12 @@
       <c r="C68" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D68" s="1"/>
-      <c r="E68" s="1"/>
+      <c r="D68" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E68" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F68" s="1"/>
       <c r="G68" s="1"/>
       <c r="H68" s="1"/>
@@ -19282,8 +19566,12 @@
       <c r="C69" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D69" s="1"/>
-      <c r="E69" s="1"/>
+      <c r="D69" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E69" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F69" s="1"/>
       <c r="G69" s="1"/>
       <c r="H69" s="1"/>
@@ -19313,8 +19601,12 @@
       <c r="C70" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D70" s="1"/>
-      <c r="E70" s="1"/>
+      <c r="D70" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F70" s="1"/>
       <c r="G70" s="1"/>
       <c r="H70" s="1"/>
@@ -19344,8 +19636,12 @@
       <c r="C71" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D71" s="1"/>
-      <c r="E71" s="1"/>
+      <c r="D71" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F71" s="1"/>
       <c r="G71" s="1"/>
       <c r="H71" s="1"/>
@@ -19375,8 +19671,12 @@
       <c r="C72" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D72" s="1"/>
-      <c r="E72" s="1"/>
+      <c r="D72" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>735</v>
+      </c>
       <c r="F72" s="1"/>
       <c r="G72" s="1"/>
       <c r="H72" s="1"/>
@@ -42279,42 +42579,48 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:B1000"/>
+  <dimension ref="A1:C1000"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="26" width="10.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.75" customHeight="1">
+    <row r="1" spans="1:3" ht="15.75" customHeight="1">
       <c r="A1" s="12" t="s">
         <v>180</v>
       </c>
       <c r="B1" s="12" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" ht="15.75" customHeight="1">
+      <c r="C1" s="18" t="s">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15.75" customHeight="1">
       <c r="A2" s="12" t="s">
         <v>181</v>
       </c>
-      <c r="B2" s="12" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="4" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="5" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="6" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="7" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="8" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="9" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="10" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="11" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="12" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="13" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="14" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="15" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="16" spans="1:2" ht="15.75" customHeight="1"/>
+      <c r="B2" s="18" t="s">
+        <v>734</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="4" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="5" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="6" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="7" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="8" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="9" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="10" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="11" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="12" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="13" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="14" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="15" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="16" spans="1:3" ht="15.75" customHeight="1"/>
     <row r="17" ht="15.75" customHeight="1"/>
     <row r="18" ht="15.75" customHeight="1"/>
     <row r="19" ht="15.75" customHeight="1"/>
@@ -43315,15 +43621,15 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15.75" customHeight="1">
       <c r="A1" s="12" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="15.75" customHeight="1">
       <c r="A2" s="12" t="s">
+        <v>183</v>
+      </c>
+      <c r="B2" s="12" t="s">
         <v>184</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15.75" customHeight="1"/>
@@ -44343,10 +44649,10 @@
   <sheetData>
     <row r="1" spans="1:4" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>186</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>187</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -44361,13 +44667,13 @@
         <v>ahd_screening</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>189</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15.75" customHeight="1">
@@ -50381,77 +50687,77 @@
   <sheetData>
     <row r="1" spans="1:9" ht="15.75" customHeight="1">
       <c r="A1" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="B1" s="15" t="s">
         <v>191</v>
       </c>
-      <c r="B1" s="15" t="s">
+      <c r="C1" s="15" t="s">
         <v>192</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="D1" s="15" t="s">
         <v>193</v>
       </c>
-      <c r="D1" s="15" t="s">
+      <c r="E1" s="15" t="s">
         <v>194</v>
       </c>
-      <c r="E1" s="15" t="s">
+      <c r="F1" s="15" t="s">
         <v>195</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="G1" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="H1" s="15" t="s">
         <v>197</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="I1" s="15" t="s">
         <v>198</v>
-      </c>
-      <c r="I1" s="15" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="15.75" customHeight="1">
       <c r="A2" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="B2" s="12" t="s">
         <v>200</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="C2" s="16" t="s">
         <v>201</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="D2" s="16" t="s">
+        <v>201</v>
+      </c>
+      <c r="E2" s="17" t="s">
         <v>202</v>
       </c>
-      <c r="D2" s="16" t="s">
-        <v>202</v>
-      </c>
-      <c r="E2" s="17" t="s">
+      <c r="F2" s="12" t="s">
         <v>203</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>204</v>
       </c>
       <c r="G2" s="12" t="s">
         <v>179</v>
       </c>
       <c r="H2" s="12" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="I2" s="12" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="15.75" customHeight="1">
       <c r="A3" s="12" t="s">
+        <v>205</v>
+      </c>
+      <c r="B3" s="12" t="s">
         <v>206</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="C3" s="12" t="s">
         <v>207</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>208</v>
       </c>
       <c r="E3" s="17" t="s">
         <v>15</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="G3" s="12" t="s">
         <v>177</v>
@@ -50460,804 +50766,804 @@
         <v>178</v>
       </c>
       <c r="I3" s="12" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.75" customHeight="1">
       <c r="A4" s="12" t="s">
+        <v>209</v>
+      </c>
+      <c r="B4" s="12" t="s">
         <v>210</v>
       </c>
-      <c r="B4" s="12" t="s">
+      <c r="C4" s="12" t="s">
         <v>211</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="E4" s="17" t="s">
         <v>212</v>
       </c>
-      <c r="E4" s="17" t="s">
+      <c r="G4" s="12" t="s">
         <v>213</v>
       </c>
-      <c r="G4" s="12" t="s">
-        <v>214</v>
-      </c>
       <c r="I4" s="12" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" customHeight="1">
       <c r="A5" s="12" t="s">
+        <v>214</v>
+      </c>
+      <c r="B5" s="12" t="s">
         <v>215</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="C5" s="12" t="s">
         <v>216</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="E5" s="17" t="s">
         <v>217</v>
       </c>
-      <c r="E5" s="17" t="s">
+      <c r="I5" s="12" t="s">
         <v>218</v>
-      </c>
-      <c r="I5" s="12" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="15.75" customHeight="1">
       <c r="A6" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="B6" s="12" t="s">
         <v>220</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="C6" s="12" t="s">
         <v>221</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="I6" s="12" t="s">
         <v>222</v>
-      </c>
-      <c r="I6" s="12" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="15.75" customHeight="1">
       <c r="A7" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="B7" s="12" t="s">
         <v>224</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="C7" s="12" t="s">
         <v>225</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="I7" s="12" t="s">
         <v>226</v>
-      </c>
-      <c r="I7" s="12" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="15.75" customHeight="1">
       <c r="A8" s="12" t="s">
+        <v>227</v>
+      </c>
+      <c r="B8" s="12" t="s">
         <v>228</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="C8" s="12" t="s">
         <v>229</v>
       </c>
-      <c r="C8" s="12" t="s">
-        <v>230</v>
-      </c>
       <c r="I8" s="12" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="15.75" customHeight="1">
       <c r="B9" s="12" t="s">
+        <v>230</v>
+      </c>
+      <c r="C9" s="12" t="s">
         <v>231</v>
       </c>
-      <c r="C9" s="12" t="s">
-        <v>232</v>
-      </c>
       <c r="I9" s="12" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15.75" customHeight="1">
       <c r="B10" s="12" t="s">
+        <v>232</v>
+      </c>
+      <c r="C10" s="12" t="s">
         <v>233</v>
       </c>
-      <c r="C10" s="12" t="s">
-        <v>234</v>
-      </c>
       <c r="I10" s="12" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="15.75" customHeight="1">
       <c r="B11" s="12" t="s">
+        <v>234</v>
+      </c>
+      <c r="C11" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="I11" s="12" t="s">
         <v>236</v>
-      </c>
-      <c r="I11" s="12" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="15.75" customHeight="1">
       <c r="B12" s="12" t="s">
+        <v>237</v>
+      </c>
+      <c r="C12" s="12" t="s">
         <v>238</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>239</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15.75" customHeight="1">
       <c r="B13" s="12" t="s">
+        <v>239</v>
+      </c>
+      <c r="C13" s="12" t="s">
         <v>240</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="15.75" customHeight="1">
       <c r="B14" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="C14" s="12" t="s">
         <v>242</v>
-      </c>
-      <c r="C14" s="12" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="15.75" customHeight="1">
       <c r="B15" s="12" t="s">
+        <v>243</v>
+      </c>
+      <c r="C15" s="12" t="s">
         <v>244</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="15.75" customHeight="1">
       <c r="B16" s="12" t="s">
+        <v>245</v>
+      </c>
+      <c r="C16" s="12" t="s">
         <v>246</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="15.75" customHeight="1">
       <c r="B17" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="C17" s="12" t="s">
         <v>248</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="15.75" customHeight="1">
       <c r="B18" s="12" t="s">
+        <v>249</v>
+      </c>
+      <c r="C18" s="12" t="s">
         <v>250</v>
-      </c>
-      <c r="C18" s="12" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="19" spans="2:3" ht="15.75" customHeight="1">
       <c r="B19" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="C19" s="12" t="s">
         <v>252</v>
-      </c>
-      <c r="C19" s="12" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="15.75" customHeight="1">
       <c r="B20" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="C20" s="12" t="s">
         <v>254</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="21" spans="2:3" ht="15.75" customHeight="1">
       <c r="B21" s="12" t="s">
+        <v>255</v>
+      </c>
+      <c r="C21" s="12" t="s">
         <v>256</v>
-      </c>
-      <c r="C21" s="12" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="22" spans="2:3" ht="15.75" customHeight="1">
       <c r="B22" s="12" t="s">
+        <v>257</v>
+      </c>
+      <c r="C22" s="12" t="s">
         <v>258</v>
-      </c>
-      <c r="C22" s="12" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="23" spans="2:3" ht="15.75" customHeight="1">
       <c r="B23" s="12" t="s">
+        <v>259</v>
+      </c>
+      <c r="C23" s="12" t="s">
         <v>260</v>
-      </c>
-      <c r="C23" s="12" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="24" spans="2:3" ht="15.75" customHeight="1">
       <c r="B24" s="12" t="s">
+        <v>261</v>
+      </c>
+      <c r="C24" s="12" t="s">
         <v>262</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="25" spans="2:3" ht="15.75" customHeight="1">
       <c r="B25" s="12" t="s">
+        <v>263</v>
+      </c>
+      <c r="C25" s="12" t="s">
         <v>264</v>
-      </c>
-      <c r="C25" s="12" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="26" spans="2:3" ht="15.75" customHeight="1">
       <c r="B26" s="12" t="s">
+        <v>265</v>
+      </c>
+      <c r="C26" s="12" t="s">
         <v>266</v>
-      </c>
-      <c r="C26" s="12" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="27" spans="2:3" ht="15.75" customHeight="1">
       <c r="B27" s="12" t="s">
+        <v>267</v>
+      </c>
+      <c r="C27" s="12" t="s">
         <v>268</v>
-      </c>
-      <c r="C27" s="12" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="28" spans="2:3" ht="15.75" customHeight="1">
       <c r="B28" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="C28" s="12" t="s">
         <v>270</v>
-      </c>
-      <c r="C28" s="12" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="29" spans="2:3" ht="15.75" customHeight="1">
       <c r="B29" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="C29" s="12" t="s">
         <v>272</v>
-      </c>
-      <c r="C29" s="12" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="30" spans="2:3" ht="15.75" customHeight="1">
       <c r="B30" s="12" t="s">
+        <v>273</v>
+      </c>
+      <c r="C30" s="12" t="s">
         <v>274</v>
-      </c>
-      <c r="C30" s="12" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="31" spans="2:3" ht="15.75" customHeight="1">
       <c r="B31" s="12" t="s">
+        <v>275</v>
+      </c>
+      <c r="C31" s="12" t="s">
         <v>276</v>
-      </c>
-      <c r="C31" s="12" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="32" spans="2:3" ht="15.75" customHeight="1">
       <c r="C32" s="12" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="33" spans="3:3" ht="15.75" customHeight="1">
       <c r="C33" s="12" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="34" spans="3:3" ht="15.75" customHeight="1">
       <c r="C34" s="12" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="35" spans="3:3" ht="15.75" customHeight="1">
       <c r="C35" s="12" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="36" spans="3:3" ht="15.75" customHeight="1">
       <c r="C36" s="12" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="37" spans="3:3" ht="15.75" customHeight="1">
       <c r="C37" s="12" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="38" spans="3:3" ht="15.75" customHeight="1">
       <c r="C38" s="12" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="39" spans="3:3" ht="15.75" customHeight="1">
       <c r="C39" s="12" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="40" spans="3:3" ht="15.75" customHeight="1">
       <c r="C40" s="12" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="41" spans="3:3" ht="15.75" customHeight="1">
       <c r="C41" s="12" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="42" spans="3:3" ht="15.75" customHeight="1">
       <c r="C42" s="12" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="43" spans="3:3" ht="15.75" customHeight="1">
       <c r="C43" s="12" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="44" spans="3:3" ht="15.75" customHeight="1">
       <c r="C44" s="12" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="45" spans="3:3" ht="15.75" customHeight="1">
       <c r="C45" s="12" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="46" spans="3:3" ht="15.75" customHeight="1">
       <c r="C46" s="12" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="47" spans="3:3" ht="15.75" customHeight="1">
       <c r="C47" s="12" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="48" spans="3:3" ht="15.75" customHeight="1">
       <c r="C48" s="12" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="49" spans="3:3" ht="15.75" customHeight="1">
       <c r="C49" s="12" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="50" spans="3:3" ht="15.75" customHeight="1">
       <c r="C50" s="12" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="51" spans="3:3" ht="15.75" customHeight="1">
       <c r="C51" s="12" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="52" spans="3:3" ht="15.75" customHeight="1">
       <c r="C52" s="12" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="53" spans="3:3" ht="15.75" customHeight="1">
       <c r="C53" s="12" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="54" spans="3:3" ht="15.75" customHeight="1">
       <c r="C54" s="12" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="55" spans="3:3" ht="15.75" customHeight="1">
       <c r="C55" s="12" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="56" spans="3:3" ht="15.75" customHeight="1">
       <c r="C56" s="12" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="57" spans="3:3" ht="15.75" customHeight="1">
       <c r="C57" s="12" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="58" spans="3:3" ht="15.75" customHeight="1">
       <c r="C58" s="12" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="59" spans="3:3" ht="15.75" customHeight="1">
       <c r="C59" s="12" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="60" spans="3:3" ht="15.75" customHeight="1">
       <c r="C60" s="12" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="61" spans="3:3" ht="15.75" customHeight="1">
       <c r="C61" s="12" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="62" spans="3:3" ht="15.75" customHeight="1">
       <c r="C62" s="12" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="63" spans="3:3" ht="15.75" customHeight="1">
       <c r="C63" s="12" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="64" spans="3:3" ht="15.75" customHeight="1">
       <c r="C64" s="12" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="65" spans="3:3" ht="15.75" customHeight="1">
       <c r="C65" s="12" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="66" spans="3:3" ht="15.75" customHeight="1">
       <c r="C66" s="12" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="67" spans="3:3" ht="15.75" customHeight="1">
       <c r="C67" s="12" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="68" spans="3:3" ht="15.75" customHeight="1">
       <c r="C68" s="12" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="69" spans="3:3" ht="15.75" customHeight="1">
       <c r="C69" s="12" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="70" spans="3:3" ht="15.75" customHeight="1">
       <c r="C70" s="12" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="71" spans="3:3" ht="15.75" customHeight="1">
       <c r="C71" s="12" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="72" spans="3:3" ht="15.75" customHeight="1">
       <c r="C72" s="12" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="73" spans="3:3" ht="15.75" customHeight="1">
       <c r="C73" s="12" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="74" spans="3:3" ht="15.75" customHeight="1">
       <c r="C74" s="12" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="75" spans="3:3" ht="15.75" customHeight="1">
       <c r="C75" s="12" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="76" spans="3:3" ht="15.75" customHeight="1">
       <c r="C76" s="12" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="77" spans="3:3" ht="15.75" customHeight="1">
       <c r="C77" s="12" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="78" spans="3:3" ht="15.75" customHeight="1">
       <c r="C78" s="12" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="79" spans="3:3" ht="15.75" customHeight="1">
       <c r="C79" s="12" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="80" spans="3:3" ht="15.75" customHeight="1">
       <c r="C80" s="12" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="81" spans="3:3" ht="15.75" customHeight="1">
       <c r="C81" s="12" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="82" spans="3:3" ht="15.75" customHeight="1">
       <c r="C82" s="12" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="83" spans="3:3" ht="15.75" customHeight="1">
       <c r="C83" s="12" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="84" spans="3:3" ht="15.75" customHeight="1">
       <c r="C84" s="12" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="85" spans="3:3" ht="15.75" customHeight="1">
       <c r="C85" s="12" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="86" spans="3:3" ht="15.75" customHeight="1">
       <c r="C86" s="12" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="87" spans="3:3" ht="15.75" customHeight="1">
       <c r="C87" s="12" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="88" spans="3:3" ht="15.75" customHeight="1">
       <c r="C88" s="12" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="89" spans="3:3" ht="15.75" customHeight="1">
       <c r="C89" s="12" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="90" spans="3:3" ht="15.75" customHeight="1">
       <c r="C90" s="12" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="91" spans="3:3" ht="15.75" customHeight="1">
       <c r="C91" s="12" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="92" spans="3:3" ht="15.75" customHeight="1">
       <c r="C92" s="12" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="93" spans="3:3" ht="15.75" customHeight="1">
       <c r="C93" s="12" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="94" spans="3:3" ht="15.75" customHeight="1">
       <c r="C94" s="12" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="95" spans="3:3" ht="15.75" customHeight="1">
       <c r="C95" s="12" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="96" spans="3:3" ht="15.75" customHeight="1">
       <c r="C96" s="12" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="97" spans="3:3" ht="15.75" customHeight="1">
       <c r="C97" s="12" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="98" spans="3:3" ht="15.75" customHeight="1">
       <c r="C98" s="12" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="99" spans="3:3" ht="15.75" customHeight="1">
       <c r="C99" s="12" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="100" spans="3:3" ht="15.75" customHeight="1">
       <c r="C100" s="12" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="101" spans="3:3" ht="15.75" customHeight="1">
       <c r="C101" s="12" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="102" spans="3:3" ht="15.75" customHeight="1">
       <c r="C102" s="12" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="103" spans="3:3" ht="15.75" customHeight="1">
       <c r="C103" s="12" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="104" spans="3:3" ht="15.75" customHeight="1">
       <c r="C104" s="12" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="105" spans="3:3" ht="15.75" customHeight="1">
       <c r="C105" s="12" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="106" spans="3:3" ht="15.75" customHeight="1">
       <c r="C106" s="12" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="107" spans="3:3" ht="15.75" customHeight="1">
       <c r="C107" s="12" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="108" spans="3:3" ht="15.75" customHeight="1">
       <c r="C108" s="12" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="109" spans="3:3" ht="15.75" customHeight="1">
       <c r="C109" s="12" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="110" spans="3:3" ht="15.75" customHeight="1">
       <c r="C110" s="12" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="111" spans="3:3" ht="15.75" customHeight="1">
       <c r="C111" s="12" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="112" spans="3:3" ht="15.75" customHeight="1">
       <c r="C112" s="12" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="113" spans="3:3" ht="15.75" customHeight="1">
       <c r="C113" s="12" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="114" spans="3:3" ht="15.75" customHeight="1">
       <c r="C114" s="12" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="115" spans="3:3" ht="15.75" customHeight="1">
       <c r="C115" s="12" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="116" spans="3:3" ht="15.75" customHeight="1">
       <c r="C116" s="12" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="117" spans="3:3" ht="15.75" customHeight="1">
       <c r="C117" s="12" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="118" spans="3:3" ht="15.75" customHeight="1">
       <c r="C118" s="12" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="119" spans="3:3" ht="15.75" customHeight="1">
       <c r="C119" s="12" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="120" spans="3:3" ht="15.75" customHeight="1">
       <c r="C120" s="12" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="121" spans="3:3" ht="15.75" customHeight="1">
       <c r="C121" s="12" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="122" spans="3:3" ht="15.75" customHeight="1">
       <c r="C122" s="12" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="123" spans="3:3" ht="15.75" customHeight="1">
       <c r="C123" s="12" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="124" spans="3:3" ht="15.75" customHeight="1">
       <c r="C124" s="12" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="125" spans="3:3" ht="15.75" customHeight="1">
       <c r="C125" s="12" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="126" spans="3:3" ht="15.75" customHeight="1">
       <c r="C126" s="12" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="127" spans="3:3" ht="15.75" customHeight="1">
       <c r="C127" s="12" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="128" spans="3:3" ht="15.75" customHeight="1">
       <c r="C128" s="12" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="129" spans="3:3" ht="15.75" customHeight="1">
       <c r="C129" s="12" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="130" spans="3:3" ht="15.75" customHeight="1">
       <c r="C130" s="12" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="131" spans="3:3" ht="15.75" customHeight="1">
       <c r="C131" s="12" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="132" spans="3:3" ht="15.75" customHeight="1">
       <c r="C132" s="12" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="133" spans="3:3" ht="15.75" customHeight="1">
       <c r="C133" s="12" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="134" spans="3:3" ht="15.75" customHeight="1">
       <c r="C134" s="12" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="135" spans="3:3" ht="15.75" customHeight="1">
       <c r="C135" s="12" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="136" spans="3:3" ht="15.75" customHeight="1">
       <c r="C136" s="12" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="137" spans="3:3" ht="15.75" customHeight="1">
@@ -51267,122 +51573,122 @@
     </row>
     <row r="138" spans="3:3" ht="15.75" customHeight="1">
       <c r="C138" s="12" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="139" spans="3:3" ht="15.75" customHeight="1">
       <c r="C139" s="12" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="140" spans="3:3" ht="15.75" customHeight="1">
       <c r="C140" s="12" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="141" spans="3:3" ht="15.75" customHeight="1">
       <c r="C141" s="12" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="142" spans="3:3" ht="15.75" customHeight="1">
       <c r="C142" s="12" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="143" spans="3:3" ht="15.75" customHeight="1">
       <c r="C143" s="12" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="144" spans="3:3" ht="15.75" customHeight="1">
       <c r="C144" s="12" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="145" spans="3:3" ht="15.75" customHeight="1">
       <c r="C145" s="12" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="146" spans="3:3" ht="15.75" customHeight="1">
       <c r="C146" s="12" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="147" spans="3:3" ht="15.75" customHeight="1">
       <c r="C147" s="12" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="148" spans="3:3" ht="15.75" customHeight="1">
       <c r="C148" s="12" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="149" spans="3:3" ht="15.75" customHeight="1">
       <c r="C149" s="12" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="150" spans="3:3" ht="15.75" customHeight="1">
       <c r="C150" s="12" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="151" spans="3:3" ht="15.75" customHeight="1">
       <c r="C151" s="12" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="152" spans="3:3" ht="15.75" customHeight="1">
       <c r="C152" s="12" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="153" spans="3:3" ht="15.75" customHeight="1">
       <c r="C153" s="12" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="154" spans="3:3" ht="15.75" customHeight="1">
       <c r="C154" s="12" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="155" spans="3:3" ht="15.75" customHeight="1">
       <c r="C155" s="12" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="156" spans="3:3" ht="15.75" customHeight="1">
       <c r="C156" s="12" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="157" spans="3:3" ht="15.75" customHeight="1">
       <c r="C157" s="12" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="158" spans="3:3" ht="15.75" customHeight="1">
       <c r="C158" s="12" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="159" spans="3:3" ht="15.75" customHeight="1">
       <c r="C159" s="12" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="160" spans="3:3" ht="15.75" customHeight="1">
       <c r="C160" s="12" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="161" spans="3:3" ht="15.75" customHeight="1">
       <c r="C161" s="12" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="162" spans="3:3" ht="15.75" customHeight="1">
@@ -51392,852 +51698,852 @@
     </row>
     <row r="163" spans="3:3" ht="15.75" customHeight="1">
       <c r="C163" s="12" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="164" spans="3:3" ht="15.75" customHeight="1">
       <c r="C164" s="12" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="165" spans="3:3" ht="15.75" customHeight="1">
       <c r="C165" s="12" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="166" spans="3:3" ht="15.75" customHeight="1">
       <c r="C166" s="12" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="167" spans="3:3" ht="15.75" customHeight="1">
       <c r="C167" s="12" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="168" spans="3:3" ht="15.75" customHeight="1">
       <c r="C168" s="12" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="169" spans="3:3" ht="15.75" customHeight="1">
       <c r="C169" s="12" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="170" spans="3:3" ht="15.75" customHeight="1">
       <c r="C170" s="12" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="171" spans="3:3" ht="15.75" customHeight="1">
       <c r="C171" s="12" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="172" spans="3:3" ht="15.75" customHeight="1">
       <c r="C172" s="12" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="173" spans="3:3" ht="15.75" customHeight="1">
       <c r="C173" s="12" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="174" spans="3:3" ht="15.75" customHeight="1">
       <c r="C174" s="12" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="175" spans="3:3" ht="15.75" customHeight="1">
       <c r="C175" s="12" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="176" spans="3:3" ht="15.75" customHeight="1">
       <c r="C176" s="12" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="177" spans="3:3" ht="15.75" customHeight="1">
       <c r="C177" s="12" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="178" spans="3:3" ht="15.75" customHeight="1">
       <c r="C178" s="12" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="179" spans="3:3" ht="15.75" customHeight="1">
       <c r="C179" s="12" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="180" spans="3:3" ht="15.75" customHeight="1">
       <c r="C180" s="12" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="181" spans="3:3" ht="15.75" customHeight="1">
       <c r="C181" s="12" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="182" spans="3:3" ht="15.75" customHeight="1">
       <c r="C182" s="12" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="183" spans="3:3" ht="15.75" customHeight="1">
       <c r="C183" s="12" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="184" spans="3:3" ht="15.75" customHeight="1">
       <c r="C184" s="12" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="185" spans="3:3" ht="15.75" customHeight="1">
       <c r="C185" s="12" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="186" spans="3:3" ht="15.75" customHeight="1">
       <c r="C186" s="12" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="187" spans="3:3" ht="15.75" customHeight="1">
       <c r="C187" s="12" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="188" spans="3:3" ht="15.75" customHeight="1">
       <c r="C188" s="12" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="189" spans="3:3" ht="15.75" customHeight="1">
       <c r="C189" s="12" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="190" spans="3:3" ht="15.75" customHeight="1">
       <c r="C190" s="12" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="191" spans="3:3" ht="15.75" customHeight="1">
       <c r="C191" s="12" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="192" spans="3:3" ht="15.75" customHeight="1">
       <c r="C192" s="12" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="193" spans="3:3" ht="15.75" customHeight="1">
       <c r="C193" s="12" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="194" spans="3:3" ht="15.75" customHeight="1">
       <c r="C194" s="12" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="195" spans="3:3" ht="15.75" customHeight="1">
       <c r="C195" s="12" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="196" spans="3:3" ht="15.75" customHeight="1">
       <c r="C196" s="12" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="197" spans="3:3" ht="15.75" customHeight="1">
       <c r="C197" s="12" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="198" spans="3:3" ht="15.75" customHeight="1">
       <c r="C198" s="12" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="199" spans="3:3" ht="15.75" customHeight="1">
       <c r="C199" s="12" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="200" spans="3:3" ht="15.75" customHeight="1">
       <c r="C200" s="12" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="201" spans="3:3" ht="15.75" customHeight="1">
       <c r="C201" s="12" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="202" spans="3:3" ht="15.75" customHeight="1">
       <c r="C202" s="12" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="203" spans="3:3" ht="15.75" customHeight="1">
       <c r="C203" s="12" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="204" spans="3:3" ht="15.75" customHeight="1">
       <c r="C204" s="12" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="205" spans="3:3" ht="15.75" customHeight="1">
       <c r="C205" s="12" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
     </row>
     <row r="206" spans="3:3" ht="15.75" customHeight="1">
       <c r="C206" s="12" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
     </row>
     <row r="207" spans="3:3" ht="15.75" customHeight="1">
       <c r="C207" s="12" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
     <row r="208" spans="3:3" ht="15.75" customHeight="1">
       <c r="C208" s="12" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
     </row>
     <row r="209" spans="3:3" ht="15.75" customHeight="1">
       <c r="C209" s="12" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
     </row>
     <row r="210" spans="3:3" ht="15.75" customHeight="1">
       <c r="C210" s="12" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
     </row>
     <row r="211" spans="3:3" ht="15.75" customHeight="1">
       <c r="C211" s="12" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="212" spans="3:3" ht="15.75" customHeight="1">
       <c r="C212" s="12" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
     </row>
     <row r="213" spans="3:3" ht="15.75" customHeight="1">
       <c r="C213" s="12" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="214" spans="3:3" ht="15.75" customHeight="1">
       <c r="C214" s="12" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="215" spans="3:3" ht="15.75" customHeight="1">
       <c r="C215" s="12" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="216" spans="3:3" ht="15.75" customHeight="1">
       <c r="C216" s="12" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
     </row>
     <row r="217" spans="3:3" ht="15.75" customHeight="1">
       <c r="C217" s="12" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
     </row>
     <row r="218" spans="3:3" ht="15.75" customHeight="1">
       <c r="C218" s="12" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="219" spans="3:3" ht="15.75" customHeight="1">
       <c r="C219" s="12" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="220" spans="3:3" ht="15.75" customHeight="1">
       <c r="C220" s="12" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
     </row>
     <row r="221" spans="3:3" ht="15.75" customHeight="1">
       <c r="C221" s="12" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
     </row>
     <row r="222" spans="3:3" ht="15.75" customHeight="1">
       <c r="C222" s="12" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
     </row>
     <row r="223" spans="3:3" ht="15.75" customHeight="1">
       <c r="C223" s="12" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
     </row>
     <row r="224" spans="3:3" ht="15.75" customHeight="1">
       <c r="C224" s="12" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
     </row>
     <row r="225" spans="3:3" ht="15.75" customHeight="1">
       <c r="C225" s="12" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
     </row>
     <row r="226" spans="3:3" ht="15.75" customHeight="1">
       <c r="C226" s="12" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
     </row>
     <row r="227" spans="3:3" ht="15.75" customHeight="1">
       <c r="C227" s="12" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
     </row>
     <row r="228" spans="3:3" ht="15.75" customHeight="1">
       <c r="C228" s="12" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
     </row>
     <row r="229" spans="3:3" ht="15.75" customHeight="1">
       <c r="C229" s="12" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="230" spans="3:3" ht="15.75" customHeight="1">
       <c r="C230" s="12" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
     </row>
     <row r="231" spans="3:3" ht="15.75" customHeight="1">
       <c r="C231" s="12" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
     </row>
     <row r="232" spans="3:3" ht="15.75" customHeight="1">
       <c r="C232" s="12" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="233" spans="3:3" ht="15.75" customHeight="1">
       <c r="C233" s="12" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="234" spans="3:3" ht="15.75" customHeight="1">
       <c r="C234" s="12" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="235" spans="3:3" ht="15.75" customHeight="1">
       <c r="C235" s="12" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
     </row>
     <row r="236" spans="3:3" ht="15.75" customHeight="1">
       <c r="C236" s="12" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
     </row>
     <row r="237" spans="3:3" ht="15.75" customHeight="1">
       <c r="C237" s="12" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="238" spans="3:3" ht="15.75" customHeight="1">
       <c r="C238" s="12" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
     </row>
     <row r="239" spans="3:3" ht="15.75" customHeight="1">
       <c r="C239" s="12" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
     </row>
     <row r="240" spans="3:3" ht="15.75" customHeight="1">
       <c r="C240" s="12" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
     </row>
     <row r="241" spans="3:3" ht="15.75" customHeight="1">
       <c r="C241" s="12" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
     </row>
     <row r="242" spans="3:3" ht="15.75" customHeight="1">
       <c r="C242" s="12" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
     </row>
     <row r="243" spans="3:3" ht="15.75" customHeight="1">
       <c r="C243" s="12" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
     </row>
     <row r="244" spans="3:3" ht="15.75" customHeight="1">
       <c r="C244" s="12" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
     </row>
     <row r="245" spans="3:3" ht="15.75" customHeight="1">
       <c r="C245" s="12" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
     </row>
     <row r="246" spans="3:3" ht="15.75" customHeight="1">
       <c r="C246" s="12" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="247" spans="3:3" ht="15.75" customHeight="1">
       <c r="C247" s="12" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
     </row>
     <row r="248" spans="3:3" ht="15.75" customHeight="1">
       <c r="C248" s="12" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
     </row>
     <row r="249" spans="3:3" ht="15.75" customHeight="1">
       <c r="C249" s="12" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="250" spans="3:3" ht="15.75" customHeight="1">
       <c r="C250" s="12" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
     </row>
     <row r="251" spans="3:3" ht="15.75" customHeight="1">
       <c r="C251" s="12" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
     </row>
     <row r="252" spans="3:3" ht="15.75" customHeight="1">
       <c r="C252" s="12" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
     </row>
     <row r="253" spans="3:3" ht="15.75" customHeight="1">
       <c r="C253" s="12" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
     </row>
     <row r="254" spans="3:3" ht="15.75" customHeight="1">
       <c r="C254" s="12" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
     </row>
     <row r="255" spans="3:3" ht="15.75" customHeight="1">
       <c r="C255" s="12" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
     </row>
     <row r="256" spans="3:3" ht="15.75" customHeight="1">
       <c r="C256" s="12" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="257" spans="3:3" ht="15.75" customHeight="1">
       <c r="C257" s="12" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
     </row>
     <row r="258" spans="3:3" ht="15.75" customHeight="1">
       <c r="C258" s="12" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="259" spans="3:3" ht="15.75" customHeight="1">
       <c r="C259" s="12" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
     </row>
     <row r="260" spans="3:3" ht="15.75" customHeight="1">
       <c r="C260" s="12" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
     </row>
     <row r="261" spans="3:3" ht="15.75" customHeight="1">
       <c r="C261" s="12" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
     <row r="262" spans="3:3" ht="15.75" customHeight="1">
       <c r="C262" s="12" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="263" spans="3:3" ht="15.75" customHeight="1">
       <c r="C263" s="12" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
     <row r="264" spans="3:3" ht="15.75" customHeight="1">
       <c r="C264" s="12" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
     </row>
     <row r="265" spans="3:3" ht="15.75" customHeight="1">
       <c r="C265" s="12" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
     </row>
     <row r="266" spans="3:3" ht="15.75" customHeight="1">
       <c r="C266" s="12" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="267" spans="3:3" ht="15.75" customHeight="1">
       <c r="C267" s="12" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
     </row>
     <row r="268" spans="3:3" ht="15.75" customHeight="1">
       <c r="C268" s="12" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
     </row>
     <row r="269" spans="3:3" ht="15.75" customHeight="1">
       <c r="C269" s="12" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
     </row>
     <row r="270" spans="3:3" ht="15.75" customHeight="1">
       <c r="C270" s="12" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
     </row>
     <row r="271" spans="3:3" ht="15.75" customHeight="1">
       <c r="C271" s="12" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
     </row>
     <row r="272" spans="3:3" ht="15.75" customHeight="1">
       <c r="C272" s="12" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
     </row>
     <row r="273" spans="3:3" ht="15.75" customHeight="1">
       <c r="C273" s="12" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
     </row>
     <row r="274" spans="3:3" ht="15.75" customHeight="1">
       <c r="C274" s="12" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="275" spans="3:3" ht="15.75" customHeight="1">
       <c r="C275" s="12" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="276" spans="3:3" ht="15.75" customHeight="1">
       <c r="C276" s="12" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
     </row>
     <row r="277" spans="3:3" ht="15.75" customHeight="1">
       <c r="C277" s="12" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
     </row>
     <row r="278" spans="3:3" ht="15.75" customHeight="1">
       <c r="C278" s="12" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="279" spans="3:3" ht="15.75" customHeight="1">
       <c r="C279" s="12" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
     </row>
     <row r="280" spans="3:3" ht="15.75" customHeight="1">
       <c r="C280" s="12" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
     </row>
     <row r="281" spans="3:3" ht="15.75" customHeight="1">
       <c r="C281" s="12" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
     </row>
     <row r="282" spans="3:3" ht="15.75" customHeight="1">
       <c r="C282" s="12" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
     </row>
     <row r="283" spans="3:3" ht="15.75" customHeight="1">
       <c r="C283" s="12" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
     </row>
     <row r="284" spans="3:3" ht="15.75" customHeight="1">
       <c r="C284" s="12" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
     </row>
     <row r="285" spans="3:3" ht="15.75" customHeight="1">
       <c r="C285" s="12" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
     </row>
     <row r="286" spans="3:3" ht="15.75" customHeight="1">
       <c r="C286" s="12" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
     </row>
     <row r="287" spans="3:3" ht="15.75" customHeight="1">
       <c r="C287" s="12" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
     </row>
     <row r="288" spans="3:3" ht="15.75" customHeight="1">
       <c r="C288" s="12" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
     </row>
     <row r="289" spans="3:3" ht="15.75" customHeight="1">
       <c r="C289" s="12" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
     </row>
     <row r="290" spans="3:3" ht="15.75" customHeight="1">
       <c r="C290" s="12" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
     </row>
     <row r="291" spans="3:3" ht="15.75" customHeight="1">
       <c r="C291" s="12" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
     </row>
     <row r="292" spans="3:3" ht="15.75" customHeight="1">
       <c r="C292" s="12" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
     </row>
     <row r="293" spans="3:3" ht="15.75" customHeight="1">
       <c r="C293" s="12" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
     </row>
     <row r="294" spans="3:3" ht="15.75" customHeight="1">
       <c r="C294" s="12" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
     </row>
     <row r="295" spans="3:3" ht="15.75" customHeight="1">
       <c r="C295" s="12" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
     </row>
     <row r="296" spans="3:3" ht="15.75" customHeight="1">
       <c r="C296" s="12" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
     </row>
     <row r="297" spans="3:3" ht="15.75" customHeight="1">
       <c r="C297" s="12" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
     </row>
     <row r="298" spans="3:3" ht="15.75" customHeight="1">
       <c r="C298" s="12" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
     </row>
     <row r="299" spans="3:3" ht="15.75" customHeight="1">
       <c r="C299" s="12" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
     </row>
     <row r="300" spans="3:3" ht="15.75" customHeight="1">
       <c r="C300" s="12" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
     </row>
     <row r="301" spans="3:3" ht="15.75" customHeight="1">
       <c r="C301" s="12" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
     </row>
     <row r="302" spans="3:3" ht="15.75" customHeight="1">
       <c r="C302" s="12" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
     </row>
     <row r="303" spans="3:3" ht="15.75" customHeight="1">
       <c r="C303" s="12" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
     </row>
     <row r="304" spans="3:3" ht="15.75" customHeight="1">
       <c r="C304" s="12" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
     </row>
     <row r="305" spans="3:3" ht="15.75" customHeight="1">
       <c r="C305" s="12" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
     </row>
     <row r="306" spans="3:3" ht="15.75" customHeight="1">
       <c r="C306" s="12" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
     </row>
     <row r="307" spans="3:3" ht="15.75" customHeight="1">
       <c r="C307" s="12" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
     </row>
     <row r="308" spans="3:3" ht="15.75" customHeight="1">
       <c r="C308" s="12" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
     </row>
     <row r="309" spans="3:3" ht="15.75" customHeight="1">
       <c r="C309" s="12" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
     </row>
     <row r="310" spans="3:3" ht="15.75" customHeight="1">
       <c r="C310" s="12" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
     </row>
     <row r="311" spans="3:3" ht="15.75" customHeight="1">
       <c r="C311" s="12" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
     </row>
     <row r="312" spans="3:3" ht="15.75" customHeight="1">
       <c r="C312" s="12" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
     </row>
     <row r="313" spans="3:3" ht="15.75" customHeight="1">
       <c r="C313" s="12" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="314" spans="3:3" ht="15.75" customHeight="1">
       <c r="C314" s="12" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="315" spans="3:3" ht="15.75" customHeight="1">
       <c r="C315" s="12" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
     </row>
     <row r="316" spans="3:3" ht="15.75" customHeight="1">
       <c r="C316" s="12" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
     </row>
     <row r="317" spans="3:3" ht="15.75" customHeight="1">
       <c r="C317" s="12" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
     </row>
     <row r="318" spans="3:3" ht="15.75" customHeight="1">
       <c r="C318" s="12" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
     </row>
     <row r="319" spans="3:3" ht="15.75" customHeight="1">
       <c r="C319" s="12" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
     </row>
     <row r="320" spans="3:3" ht="15.75" customHeight="1">
       <c r="C320" s="12" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="321" spans="3:3" ht="15.75" customHeight="1">
       <c r="C321" s="12" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="322" spans="3:3" ht="15.75" customHeight="1">
       <c r="C322" s="12" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="323" spans="3:3" ht="15.75" customHeight="1">
       <c r="C323" s="12" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="324" spans="3:3" ht="15.75" customHeight="1">
       <c r="C324" s="12" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="325" spans="3:3" ht="15.75" customHeight="1">
       <c r="C325" s="12" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="326" spans="3:3" ht="15.75" customHeight="1">
       <c r="C326" s="12" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="327" spans="3:3" ht="15.75" customHeight="1">
       <c r="C327" s="12" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
     </row>
     <row r="328" spans="3:3" ht="15.75" customHeight="1">
       <c r="C328" s="12" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
     </row>
     <row r="329" spans="3:3" ht="15.75" customHeight="1">
       <c r="C329" s="12" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
     </row>
     <row r="330" spans="3:3" ht="15.75" customHeight="1">
       <c r="C330" s="12" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
     </row>
     <row r="331" spans="3:3" ht="15.75" customHeight="1">
       <c r="C331" s="12" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="332" spans="3:3" ht="15.75" customHeight="1">
       <c r="C332" s="12" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
     <row r="333" spans="3:3" ht="15.75" customHeight="1">
@@ -52247,97 +52553,97 @@
     </row>
     <row r="334" spans="3:3" ht="15.75" customHeight="1">
       <c r="C334" s="12" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
     </row>
     <row r="335" spans="3:3" ht="15.75" customHeight="1">
       <c r="C335" s="12" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
     </row>
     <row r="336" spans="3:3" ht="15.75" customHeight="1">
       <c r="C336" s="12" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
     </row>
     <row r="337" spans="3:3" ht="15.75" customHeight="1">
       <c r="C337" s="12" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
     </row>
     <row r="338" spans="3:3" ht="15.75" customHeight="1">
       <c r="C338" s="12" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="339" spans="3:3" ht="15.75" customHeight="1">
       <c r="C339" s="12" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="340" spans="3:3" ht="15.75" customHeight="1">
       <c r="C340" s="12" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
     </row>
     <row r="341" spans="3:3" ht="15.75" customHeight="1">
       <c r="C341" s="12" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
     </row>
     <row r="342" spans="3:3" ht="15.75" customHeight="1">
       <c r="C342" s="12" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
     </row>
     <row r="343" spans="3:3" ht="15.75" customHeight="1">
       <c r="C343" s="12" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
     </row>
     <row r="344" spans="3:3" ht="15.75" customHeight="1">
       <c r="C344" s="12" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
     </row>
     <row r="345" spans="3:3" ht="15.75" customHeight="1">
       <c r="C345" s="12" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
     </row>
     <row r="346" spans="3:3" ht="15.75" customHeight="1">
       <c r="C346" s="12" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="347" spans="3:3" ht="15.75" customHeight="1">
       <c r="C347" s="12" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
     </row>
     <row r="348" spans="3:3" ht="15.75" customHeight="1">
       <c r="C348" s="12" t="s">
-        <v>591</v>
+        <v>590</v>
       </c>
     </row>
     <row r="349" spans="3:3" ht="15.75" customHeight="1">
       <c r="C349" s="12" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
     </row>
     <row r="350" spans="3:3" ht="15.75" customHeight="1">
       <c r="C350" s="12" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
     </row>
     <row r="351" spans="3:3" ht="15.75" customHeight="1">
       <c r="C351" s="12" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
     </row>
     <row r="352" spans="3:3" ht="15.75" customHeight="1">
       <c r="C352" s="12" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
     </row>
     <row r="353" spans="3:3" ht="15.75" customHeight="1">
@@ -52347,292 +52653,292 @@
     </row>
     <row r="354" spans="3:3" ht="15.75" customHeight="1">
       <c r="C354" s="12" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
     </row>
     <row r="355" spans="3:3" ht="15.75" customHeight="1">
       <c r="C355" s="12" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
     </row>
     <row r="356" spans="3:3" ht="15.75" customHeight="1">
       <c r="C356" s="12" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
     </row>
     <row r="357" spans="3:3" ht="15.75" customHeight="1">
       <c r="C357" s="12" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
     </row>
     <row r="358" spans="3:3" ht="15.75" customHeight="1">
       <c r="C358" s="12" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
     </row>
     <row r="359" spans="3:3" ht="15.75" customHeight="1">
       <c r="C359" s="12" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
     </row>
     <row r="360" spans="3:3" ht="15.75" customHeight="1">
       <c r="C360" s="12" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="361" spans="3:3" ht="15.75" customHeight="1">
       <c r="C361" s="12" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
     </row>
     <row r="362" spans="3:3" ht="15.75" customHeight="1">
       <c r="C362" s="12" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
     </row>
     <row r="363" spans="3:3" ht="15.75" customHeight="1">
       <c r="C363" s="12" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
     </row>
     <row r="364" spans="3:3" ht="15.75" customHeight="1">
       <c r="C364" s="12" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
     </row>
     <row r="365" spans="3:3" ht="15.75" customHeight="1">
       <c r="C365" s="12" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="366" spans="3:3" ht="15.75" customHeight="1">
       <c r="C366" s="12" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
     </row>
     <row r="367" spans="3:3" ht="15.75" customHeight="1">
       <c r="C367" s="12" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
     </row>
     <row r="368" spans="3:3" ht="15.75" customHeight="1">
       <c r="C368" s="12" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
     </row>
     <row r="369" spans="3:3" ht="15.75" customHeight="1">
       <c r="C369" s="12" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
     </row>
     <row r="370" spans="3:3" ht="15.75" customHeight="1">
       <c r="C370" s="12" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
     </row>
     <row r="371" spans="3:3" ht="15.75" customHeight="1">
       <c r="C371" s="12" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
     </row>
     <row r="372" spans="3:3" ht="15.75" customHeight="1">
       <c r="C372" s="12" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
     </row>
     <row r="373" spans="3:3" ht="15.75" customHeight="1">
       <c r="C373" s="12" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
     </row>
     <row r="374" spans="3:3" ht="15.75" customHeight="1">
       <c r="C374" s="12" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
     </row>
     <row r="375" spans="3:3" ht="15.75" customHeight="1">
       <c r="C375" s="12" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
     </row>
     <row r="376" spans="3:3" ht="15.75" customHeight="1">
       <c r="C376" s="12" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
     </row>
     <row r="377" spans="3:3" ht="15.75" customHeight="1">
       <c r="C377" s="12" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
     </row>
     <row r="378" spans="3:3" ht="15.75" customHeight="1">
       <c r="C378" s="12" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
     </row>
     <row r="379" spans="3:3" ht="15.75" customHeight="1">
       <c r="C379" s="12" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
     </row>
     <row r="380" spans="3:3" ht="15.75" customHeight="1">
       <c r="C380" s="12" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
     </row>
     <row r="381" spans="3:3" ht="15.75" customHeight="1">
       <c r="C381" s="12" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
     </row>
     <row r="382" spans="3:3" ht="15.75" customHeight="1">
       <c r="C382" s="12" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
     </row>
     <row r="383" spans="3:3" ht="15.75" customHeight="1">
       <c r="C383" s="12" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="384" spans="3:3" ht="15.75" customHeight="1">
       <c r="C384" s="12" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
     </row>
     <row r="385" spans="3:3" ht="15.75" customHeight="1">
       <c r="C385" s="12" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
     </row>
     <row r="386" spans="3:3" ht="15.75" customHeight="1">
       <c r="C386" s="12" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
     </row>
     <row r="387" spans="3:3" ht="15.75" customHeight="1">
       <c r="C387" s="12" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="388" spans="3:3" ht="15.75" customHeight="1">
       <c r="C388" s="12" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
     </row>
     <row r="389" spans="3:3" ht="15.75" customHeight="1">
       <c r="C389" s="12" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
     </row>
     <row r="390" spans="3:3" ht="15.75" customHeight="1">
       <c r="C390" s="12" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
     </row>
     <row r="391" spans="3:3" ht="15.75" customHeight="1">
       <c r="C391" s="12" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
     </row>
     <row r="392" spans="3:3" ht="15.75" customHeight="1">
       <c r="C392" s="12" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
     </row>
     <row r="393" spans="3:3" ht="15.75" customHeight="1">
       <c r="C393" s="12" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
     </row>
     <row r="394" spans="3:3" ht="15.75" customHeight="1">
       <c r="C394" s="12" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
     </row>
     <row r="395" spans="3:3" ht="15.75" customHeight="1">
       <c r="C395" s="12" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
     </row>
     <row r="396" spans="3:3" ht="15.75" customHeight="1">
       <c r="C396" s="12" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
     </row>
     <row r="397" spans="3:3" ht="15.75" customHeight="1">
       <c r="C397" s="12" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
     </row>
     <row r="398" spans="3:3" ht="15.75" customHeight="1">
       <c r="C398" s="12" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="399" spans="3:3" ht="15.75" customHeight="1">
       <c r="C399" s="12" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
     </row>
     <row r="400" spans="3:3" ht="15.75" customHeight="1">
       <c r="C400" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
     </row>
     <row r="401" spans="3:3" ht="15.75" customHeight="1">
       <c r="C401" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
     </row>
     <row r="402" spans="3:3" ht="15.75" customHeight="1">
       <c r="C402" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
     </row>
     <row r="403" spans="3:3" ht="15.75" customHeight="1">
       <c r="C403" s="12" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
     </row>
     <row r="404" spans="3:3" ht="15.75" customHeight="1">
       <c r="C404" s="12" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
     </row>
     <row r="405" spans="3:3" ht="15.75" customHeight="1">
       <c r="C405" s="12" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
     </row>
     <row r="406" spans="3:3" ht="15.75" customHeight="1">
       <c r="C406" s="12" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
     </row>
     <row r="407" spans="3:3" ht="15.75" customHeight="1">
       <c r="C407" s="12" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
     </row>
     <row r="408" spans="3:3" ht="15.75" customHeight="1">
       <c r="C408" s="12" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
     </row>
     <row r="409" spans="3:3" ht="15.75" customHeight="1">
       <c r="C409" s="12" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="410" spans="3:3" ht="15.75" customHeight="1">
       <c r="C410" s="12" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
     </row>
     <row r="411" spans="3:3" ht="15.75" customHeight="1">
       <c r="C411" s="12" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
     </row>
     <row r="412" spans="3:3" ht="15.75" customHeight="1">
@@ -52642,402 +52948,402 @@
     </row>
     <row r="413" spans="3:3" ht="15.75" customHeight="1">
       <c r="C413" s="12" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
     </row>
     <row r="414" spans="3:3" ht="15.75" customHeight="1">
       <c r="C414" s="12" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
     </row>
     <row r="415" spans="3:3" ht="15.75" customHeight="1">
       <c r="C415" s="12" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
     </row>
     <row r="416" spans="3:3" ht="15.75" customHeight="1">
       <c r="C416" s="12" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
     </row>
     <row r="417" spans="3:3" ht="15.75" customHeight="1">
       <c r="C417" s="12" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
     </row>
     <row r="418" spans="3:3" ht="15.75" customHeight="1">
       <c r="C418" s="12" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
     </row>
     <row r="419" spans="3:3" ht="15.75" customHeight="1">
       <c r="C419" s="12" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
     </row>
     <row r="420" spans="3:3" ht="15.75" customHeight="1">
       <c r="C420" s="12" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
     </row>
     <row r="421" spans="3:3" ht="15.75" customHeight="1">
       <c r="C421" s="12" t="s">
-        <v>662</v>
+        <v>661</v>
       </c>
     </row>
     <row r="422" spans="3:3" ht="15.75" customHeight="1">
       <c r="C422" s="12" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
     </row>
     <row r="423" spans="3:3" ht="15.75" customHeight="1">
       <c r="C423" s="12" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
     </row>
     <row r="424" spans="3:3" ht="15.75" customHeight="1">
       <c r="C424" s="12" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
     </row>
     <row r="425" spans="3:3" ht="15.75" customHeight="1">
       <c r="C425" s="12" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
     </row>
     <row r="426" spans="3:3" ht="15.75" customHeight="1">
       <c r="C426" s="12" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
     </row>
     <row r="427" spans="3:3" ht="15.75" customHeight="1">
       <c r="C427" s="12" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
     </row>
     <row r="428" spans="3:3" ht="15.75" customHeight="1">
       <c r="C428" s="12" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
     </row>
     <row r="429" spans="3:3" ht="15.75" customHeight="1">
       <c r="C429" s="12" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="430" spans="3:3" ht="15.75" customHeight="1">
       <c r="C430" s="12" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="431" spans="3:3" ht="15.75" customHeight="1">
       <c r="C431" s="12" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
     </row>
     <row r="432" spans="3:3" ht="15.75" customHeight="1">
       <c r="C432" s="12" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
     </row>
     <row r="433" spans="3:3" ht="15.75" customHeight="1">
       <c r="C433" s="12" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
     </row>
     <row r="434" spans="3:3" ht="15.75" customHeight="1">
       <c r="C434" s="12" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="435" spans="3:3" ht="15.75" customHeight="1">
       <c r="C435" s="12" t="s">
-        <v>676</v>
+        <v>675</v>
       </c>
     </row>
     <row r="436" spans="3:3" ht="15.75" customHeight="1">
       <c r="C436" s="12" t="s">
-        <v>677</v>
+        <v>676</v>
       </c>
     </row>
     <row r="437" spans="3:3" ht="15.75" customHeight="1">
       <c r="C437" s="12" t="s">
-        <v>678</v>
+        <v>677</v>
       </c>
     </row>
     <row r="438" spans="3:3" ht="15.75" customHeight="1">
       <c r="C438" s="12" t="s">
-        <v>679</v>
+        <v>678</v>
       </c>
     </row>
     <row r="439" spans="3:3" ht="15.75" customHeight="1">
       <c r="C439" s="12" t="s">
-        <v>680</v>
+        <v>679</v>
       </c>
     </row>
     <row r="440" spans="3:3" ht="15.75" customHeight="1">
       <c r="C440" s="12" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
     </row>
     <row r="441" spans="3:3" ht="15.75" customHeight="1">
       <c r="C441" s="12" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
     </row>
     <row r="442" spans="3:3" ht="15.75" customHeight="1">
       <c r="C442" s="12" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
     </row>
     <row r="443" spans="3:3" ht="15.75" customHeight="1">
       <c r="C443" s="12" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
     </row>
     <row r="444" spans="3:3" ht="15.75" customHeight="1">
       <c r="C444" s="12" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
     </row>
     <row r="445" spans="3:3" ht="15.75" customHeight="1">
       <c r="C445" s="12" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
     </row>
     <row r="446" spans="3:3" ht="15.75" customHeight="1">
       <c r="C446" s="12" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
     </row>
     <row r="447" spans="3:3" ht="15.75" customHeight="1">
       <c r="C447" s="12" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
     </row>
     <row r="448" spans="3:3" ht="15.75" customHeight="1">
       <c r="C448" s="12" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
     </row>
     <row r="449" spans="3:3" ht="15.75" customHeight="1">
       <c r="C449" s="12" t="s">
-        <v>690</v>
+        <v>689</v>
       </c>
     </row>
     <row r="450" spans="3:3" ht="15.75" customHeight="1">
       <c r="C450" s="12" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
     </row>
     <row r="451" spans="3:3" ht="15.75" customHeight="1">
       <c r="C451" s="12" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="452" spans="3:3" ht="15.75" customHeight="1">
       <c r="C452" s="12" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="453" spans="3:3" ht="15.75" customHeight="1">
       <c r="C453" s="12" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
     <row r="454" spans="3:3" ht="15.75" customHeight="1">
       <c r="C454" s="12" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="455" spans="3:3" ht="15.75" customHeight="1">
       <c r="C455" s="12" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
     </row>
     <row r="456" spans="3:3" ht="15.75" customHeight="1">
       <c r="C456" s="12" t="s">
-        <v>697</v>
+        <v>696</v>
       </c>
     </row>
     <row r="457" spans="3:3" ht="15.75" customHeight="1">
       <c r="C457" s="12" t="s">
-        <v>698</v>
+        <v>697</v>
       </c>
     </row>
     <row r="458" spans="3:3" ht="15.75" customHeight="1">
       <c r="C458" s="12" t="s">
-        <v>699</v>
+        <v>698</v>
       </c>
     </row>
     <row r="459" spans="3:3" ht="15.75" customHeight="1">
       <c r="C459" s="12" t="s">
-        <v>700</v>
+        <v>699</v>
       </c>
     </row>
     <row r="460" spans="3:3" ht="15.75" customHeight="1">
       <c r="C460" s="12" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
     </row>
     <row r="461" spans="3:3" ht="15.75" customHeight="1">
       <c r="C461" s="12" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="462" spans="3:3" ht="15.75" customHeight="1">
       <c r="C462" s="12" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
     </row>
     <row r="463" spans="3:3" ht="15.75" customHeight="1">
       <c r="C463" s="12" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
     </row>
     <row r="464" spans="3:3" ht="15.75" customHeight="1">
       <c r="C464" s="12" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
     </row>
     <row r="465" spans="3:3" ht="15.75" customHeight="1">
       <c r="C465" s="12" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
     </row>
     <row r="466" spans="3:3" ht="15.75" customHeight="1">
       <c r="C466" s="12" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
     </row>
     <row r="467" spans="3:3" ht="15.75" customHeight="1">
       <c r="C467" s="12" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
     </row>
     <row r="468" spans="3:3" ht="15.75" customHeight="1">
       <c r="C468" s="12" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
     </row>
     <row r="469" spans="3:3" ht="15.75" customHeight="1">
       <c r="C469" s="12" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
     </row>
     <row r="470" spans="3:3" ht="15.75" customHeight="1">
       <c r="C470" s="12" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
     </row>
     <row r="471" spans="3:3" ht="15.75" customHeight="1">
       <c r="C471" s="12" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
     </row>
     <row r="472" spans="3:3" ht="15.75" customHeight="1">
       <c r="C472" s="12" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
     </row>
     <row r="473" spans="3:3" ht="15.75" customHeight="1">
       <c r="C473" s="12" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
     </row>
     <row r="474" spans="3:3" ht="15.75" customHeight="1">
       <c r="C474" s="12" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
     </row>
     <row r="475" spans="3:3" ht="15.75" customHeight="1">
       <c r="C475" s="12" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
     </row>
     <row r="476" spans="3:3" ht="15.75" customHeight="1">
       <c r="C476" s="12" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
     </row>
     <row r="477" spans="3:3" ht="15.75" customHeight="1">
       <c r="C477" s="12" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="478" spans="3:3" ht="15.75" customHeight="1">
       <c r="C478" s="12" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
     </row>
     <row r="479" spans="3:3" ht="15.75" customHeight="1">
       <c r="C479" s="12" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
     </row>
     <row r="480" spans="3:3" ht="15.75" customHeight="1">
       <c r="C480" s="12" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
     </row>
     <row r="481" spans="3:3" ht="15.75" customHeight="1">
       <c r="C481" s="12" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
     </row>
     <row r="482" spans="3:3" ht="15.75" customHeight="1">
       <c r="C482" s="12" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="483" spans="3:3" ht="15.75" customHeight="1">
       <c r="C483" s="12" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
     </row>
     <row r="484" spans="3:3" ht="15.75" customHeight="1">
       <c r="C484" s="12" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
     </row>
     <row r="485" spans="3:3" ht="15.75" customHeight="1">
       <c r="C485" s="12" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
     </row>
     <row r="486" spans="3:3" ht="15.75" customHeight="1">
       <c r="C486" s="12" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
     </row>
     <row r="487" spans="3:3" ht="15.75" customHeight="1">
       <c r="C487" s="12" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
     </row>
     <row r="488" spans="3:3" ht="15.75" customHeight="1">
       <c r="C488" s="12" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
     </row>
     <row r="489" spans="3:3" ht="15.75" customHeight="1">
       <c r="C489" s="12" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
     </row>
     <row r="490" spans="3:3" ht="15.75" customHeight="1">
       <c r="C490" s="12" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
     </row>
     <row r="491" spans="3:3" ht="15.75" customHeight="1">
       <c r="C491" s="12" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
     </row>
     <row r="492" spans="3:3" ht="15.75" customHeight="1">
       <c r="C492" s="12" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
     </row>
     <row r="493" spans="3:3" ht="15.75" customHeight="1"/>

</xml_diff>